<commit_message>
Publish NCT03402841, NCT03817853, NCT04004988 & NCT05176314 SoA2USDM extractions
- Extract (Layer 1) -> resolve -> consolidate for 4 protocols; regenerate index
- NCT04004988 & NCT03402841: regenerate _soa.pdf to complete SoA source
  (add tirzepatide page-11 continuation; add olaparib Table 1 screening)
- studies_protocols.xlsx: fill soa_pages for the 4; align stale soa_pages for
  NCT03637764, NCT04184622, NCT04557384 to extracted table spans
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="studies" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="protocols" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="studies" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="protocols" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -522,7 +522,6 @@
           <t>Wilsons</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>Phase 2</t>
@@ -560,7 +559,6 @@
           <t>Kidney</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Phase 1</t>
@@ -620,7 +618,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>CDISC_Pilot</t>
@@ -641,8 +638,6 @@
           <t>LZZT</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>CDISC Pilot (LZZT) synthetic study — no ClinicalTrials.gov source</t>
@@ -712,7 +707,6 @@
           <t>Diabetes</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>Phase 3</t>
@@ -750,7 +744,6 @@
           <t>Device</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>Phase 1</t>
@@ -830,7 +823,6 @@
           <t>Oncology</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>Phase 1</t>
@@ -863,7 +855,6 @@
           <t>Nektar Therapeutics</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>INSTRUCT-UC</t>
@@ -901,8 +892,6 @@
           <t>Loxo Oncology</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>Phase 1</t>
@@ -935,8 +924,6 @@
           <t>Loxo Oncology</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>Phase 1</t>
@@ -974,7 +961,6 @@
           <t>Weight</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>Phase 2</t>
@@ -1012,7 +998,6 @@
           <t>Angioedema</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>Phase 3</t>
@@ -1218,7 +1203,6 @@
           <t>Lymphoma</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>Phase 4</t>
@@ -1298,7 +1282,6 @@
           <t>Oncology</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>Phase 1/Phase 2</t>
@@ -1336,7 +1319,6 @@
           <t>Oncology</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>Phase 3</t>
@@ -1400,7 +1382,11 @@
           <t>OPINION</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>40-44</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/41/NCT03402841/Prot_002.pdf</t>
@@ -1413,8 +1399,6 @@
           <t>NCT04573309</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/09/NCT04573309/Prot_000.pdf</t>
@@ -1427,8 +1411,6 @@
           <t>NCT03283098</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/98/NCT03283098/Prot_001.pdf</t>
@@ -1446,7 +1428,6 @@
           <t>PIVOT IO 020</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/49/NCT04730349/Prot_SAP_000.pdf</t>
@@ -1464,7 +1445,6 @@
           <t>MONARCH 2</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/03/NCT02107703/Prot_000.pdf</t>
@@ -1477,8 +1457,6 @@
           <t>NCT03421379</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/79/NCT03421379/Prot_000.pdf</t>
@@ -1491,8 +1469,11 @@
           <t>NCT04004988</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>10-11</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/88/NCT04004988/Prot_000.pdf</t>
@@ -1512,7 +1493,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>19-29</t>
+          <t>18-24</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1527,10 +1508,9 @@
           <t>NCT04557384</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17-25</t>
+          <t>16-24</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1567,8 +1547,11 @@
           <t>NCT05176314</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>10-11</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/14/NCT05176314/Prot_000.pdf</t>
@@ -1581,8 +1564,6 @@
           <t>NCT05324124</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/24/NCT05324124/Prot_000.pdf</t>
@@ -1595,8 +1576,6 @@
           <t>NCT03523273</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/73/NCT03523273/Prot_SAP_000.pdf</t>
@@ -1609,8 +1588,6 @@
           <t>NCT05259917</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/17/NCT05259917/Prot_000.pdf</t>
@@ -1628,7 +1605,6 @@
           <t>STEP 1</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/35/NCT03548935/Prot_002.pdf</t>
@@ -1646,7 +1622,6 @@
           <t>STEP 4</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/87/NCT03548987/Prot_000.pdf</t>
@@ -1664,7 +1639,6 @@
           <t>STEP 5</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/30/NCT03693430/Prot_000.pdf</t>
@@ -1682,7 +1656,6 @@
           <t>MODUL</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/89/NCT02291289/Prot_000.pdf</t>
@@ -1695,8 +1668,11 @@
           <t>NCT03817853</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>100-102</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/53/NCT03817853/Prot_002.pdf</t>
@@ -1714,7 +1690,6 @@
           <t>COVACTA</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/15/NCT04320615/Prot_000.pdf</t>
@@ -1727,10 +1702,9 @@
           <t>NCT03637764</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>18-24</t>
+          <t>18-21</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1745,8 +1719,6 @@
           <t>NCT01847274</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/74/NCT01847274/Prot_000.pdf</t>

</xml_diff>

<commit_message>
Publish NCT05324124 SoA2USDM extractions
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -1564,6 +1564,11 @@
           <t>NCT05324124</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/24/NCT05324124/Prot_000.pdf</t>

</xml_diff>

<commit_message>
Publish NCT03548987 SoA2USDM extractions
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -1627,6 +1627,11 @@
           <t>STEP 4</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>8-11</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/87/NCT03548987/Prot_000.pdf</t>

</xml_diff>

<commit_message>
Publish NCT03548935 SoA2USDM extractions
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -1610,6 +1610,11 @@
           <t>STEP 1</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>8-13</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/35/NCT03548935/Prot_002.pdf</t>

</xml_diff>

<commit_message>
Publish NCT02107703 SoA2USDM extractions
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -1445,6 +1445,11 @@
           <t>MONARCH 2</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>73-78</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/03/NCT02107703/Prot_000.pdf</t>

</xml_diff>

<commit_message>
Publish NCT03421379 SoA2USDM extractions
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -1462,6 +1462,11 @@
           <t>NCT03421379</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>11-18</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/79/NCT03421379/Prot_000.pdf</t>

</xml_diff>

<commit_message>
Publish NCT03283098 SoA2USDM extractions
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -1411,6 +1411,11 @@
           <t>NCT03283098</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>32-36</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/98/NCT03283098/Prot_001.pdf</t>

</xml_diff>

<commit_message>
Publish NCT04573309 SoA2USDM extractions
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -1399,6 +1399,11 @@
           <t>NCT04573309</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>14-17</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/09/NCT04573309/Prot_000.pdf</t>

</xml_diff>

<commit_message>
Publish NCT04320615 SoA2USDM extractions
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -1725,6 +1725,11 @@
           <t>COVACTA</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>77-85</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/15/NCT04320615/Prot_000.pdf</t>

</xml_diff>

<commit_message>
Publish NCT01847274 SoA2USDM extractions (regenerated _soa.pdf: Tables 7-9)
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -1759,6 +1759,11 @@
           <t>NCT01847274</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>63-78</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/74/NCT01847274/Prot_000.pdf</t>

</xml_diff>

<commit_message>
Publish NCT04730349 SoA2USDM extractions
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -1438,6 +1438,11 @@
           <t>PIVOT IO 020</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>28-42</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/49/NCT04730349/Prot_SAP_000.pdf</t>

</xml_diff>

<commit_message>
Publish NCT05259917 SoA2USDM extractions
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -1618,6 +1618,11 @@
           <t>NCT05259917</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>17-18</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/17/NCT05259917/Prot_000.pdf</t>

</xml_diff>

<commit_message>
Publish NCT03693430 SoA2USDM extractions
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -1684,6 +1684,11 @@
           <t>STEP 5</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/30/NCT03693430/Prot_000.pdf</t>

</xml_diff>

<commit_message>
Publish NCT02291289 SoA2USDM extractions
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -1706,6 +1706,11 @@
           <t>MODUL</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>169-193</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/89/NCT02291289/Prot_000.pdf</t>

</xml_diff>

<commit_message>
usdm_data: restructure studies_protocols.xlsx + regenerate index
- studies sheet = nct_id, d4k_folder, study_acronym, study_code (real protocol study codes
  from the uncertainty reports, distinct from acronym); protocols sheet = nct_id, soa_pages,
  protocol_url. Dropped 5 unused study columns.
- Regenerate protocols/index.html: d4k Folder linked to data4knowledge/usdm_data, real study
  codes, numbered layer headers, Report column, consistent link visuals, CDISC_Pilot unlinked.
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -430,32 +430,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>lead_sponsor</t>
+          <t>study_acronym</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>therapeutic_area</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>study_acronym</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>phase</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>overall_status</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>brief_title</t>
+          <t>study_code</t>
         </is>
       </c>
     </row>
@@ -472,32 +452,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AstraZeneca</t>
+          <t>OPINION</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Oncology</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>OPINION</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Olaparib Maintenance Monotherapy in Platinum Sensitive Relapsed Non-gBRCAm Ovarian Cancer</t>
+          <t>D0816C00020</t>
         </is>
       </c>
     </row>
@@ -512,29 +472,9 @@
           <t>Alexion_NCT04573309_Wilsons</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Alexion Pharmaceuticals</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Wilsons</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Copper and Molybdenum Balance in Wilson Disease Treated With ALXN1840</t>
+          <t>ALXN1840-WD-204</t>
         </is>
       </c>
     </row>
@@ -549,29 +489,9 @@
           <t>Amgen_NCT03283098_Kidney</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Amgen</t>
-        </is>
-      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Kidney</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Phase 1</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>PK, Safety and Tolerability of AMG 416 in CKD on Hemodialysis</t>
+          <t>20140197</t>
         </is>
       </c>
     </row>
@@ -588,32 +508,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Bristol-Myers Squibb</t>
+          <t>PIVOT IO 020</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Oncology</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>PIVOT IO 020</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Phase 1/Phase 2</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Terminated</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Bempegaldesleukin + Nivolumab in Children/AYA With Recurrent or Refractory Cancer</t>
+          <t>CA045020</t>
         </is>
       </c>
     </row>
@@ -625,22 +525,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CDISC</t>
+          <t>LZZT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Pilot</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>LZZT</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>CDISC Pilot (LZZT) synthetic study — no ClinicalTrials.gov source</t>
+          <t>H2Q-MC-LZZT</t>
         </is>
       </c>
     </row>
@@ -657,32 +547,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Eli Lilly and Company</t>
+          <t>MONARCH 2</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Oncology</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>MONARCH 2</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Active, not recruiting</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Abemaciclib + Fulvestrant in HR+ HER2- Breast Cancer</t>
+          <t>I3Y-MC-JPBL</t>
         </is>
       </c>
     </row>
@@ -697,29 +567,9 @@
           <t>EliLilly_NCT03421379_Diabetes</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Eli Lilly and Company</t>
-        </is>
-      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Diabetes</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Nasal Glucagon (LY900018) in Japanese Participants With Diabetes</t>
+          <t>I8R-JE-IGBJ</t>
         </is>
       </c>
     </row>
@@ -734,29 +584,9 @@
           <t>EliLilly_NCT04004988_Device</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Eli Lilly and Company</t>
-        </is>
-      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Device</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Phase 1</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Tirzepatide by Autoinjector vs Prefilled Syringe in Healthy Participants</t>
+          <t>I8F-MC-GPGS</t>
         </is>
       </c>
     </row>
@@ -773,32 +603,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Eli Lilly and Company</t>
+          <t>SURMOUNT-1</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Diabetes</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>SURMOUNT-1</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Tirzepatide (LY3298176) in Participants With Obesity or Overweight</t>
+          <t>I8F-MC-GPHK</t>
         </is>
       </c>
     </row>
@@ -813,29 +623,9 @@
           <t>EliLilly_NCT04557384_Oncology</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Eli Lilly and Company</t>
-        </is>
-      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Oncology</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Phase 1</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Terminated</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Ramucirumab (LY3009806) SC in Participants With Advanced Cancer</t>
+          <t>I4T-MC-JVDU</t>
         </is>
       </c>
     </row>
@@ -852,27 +642,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Nektar Therapeutics</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
           <t>INSTRUCT-UC</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Terminated</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>LY3471851 in Adults With Moderately to Severely Active Ulcerative Colitis</t>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>J1P-MC-KFAH</t>
         </is>
       </c>
     </row>
@@ -887,24 +662,9 @@
           <t>EliLilly_NCT05176314</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Loxo Oncology</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Phase 1</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>DDI Study of Pirtobrutinib (LY3527727) and Rosuvastatin in Healthy Participants</t>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>J2N-MC-JZNW</t>
         </is>
       </c>
     </row>
@@ -919,24 +679,9 @@
           <t>EliLilly_NCT05324124</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Loxo Oncology</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Phase 1</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Effect of Food on Selpercatinib (LY3527723) in Healthy Participants</t>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>J2G-MC-JZPA</t>
         </is>
       </c>
     </row>
@@ -951,31 +696,6 @@
           <t>Inv_NCT03523273_Weight</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Mayo Clinic (Investigator)</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Weight</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Liraglutide 3.0 mg on Weight Loss and Gastric Functions in Obesity</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -988,29 +708,9 @@
           <t>KalVista_NCT05259917_Angioedema</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>KalVista Pharmaceuticals</t>
-        </is>
-      </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Angioedema</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>KVD900 (Sebetralstat) for On-Demand Treatment of HAE Attacks</t>
+          <t>KVD900-301</t>
         </is>
       </c>
     </row>
@@ -1027,32 +727,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>STEP 1</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Obesity</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>STEP 1</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Semaglutide 2.4 mg in Overweight or Obesity</t>
+          <t>NN9536-4373</t>
         </is>
       </c>
     </row>
@@ -1069,32 +749,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>STEP 4</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Obesity</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>STEP 4</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Semaglutide 2.4 mg After Run-in (STEP 4)</t>
+          <t>NN9536-4376</t>
         </is>
       </c>
     </row>
@@ -1111,32 +771,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>STEP 5</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Obesity</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>STEP 5</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Two-year Semaglutide 2.4 mg in Overweight or Obesity</t>
+          <t>NN9536-4378</t>
         </is>
       </c>
     </row>
@@ -1153,32 +793,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Hoffmann-La Roche</t>
+          <t>MODUL</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Oncology</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>MODUL</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Biomarker-Driven Maintenance in First-Line Metastatic Colorectal Cancer</t>
+          <t>MO29112</t>
         </is>
       </c>
     </row>
@@ -1193,29 +813,9 @@
           <t>Roche_NCT03817853_Lymphoma</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Hoffmann-La Roche</t>
-        </is>
-      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Lymphoma</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Phase 4</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Obinutuzumab Short Duration Infusion in Untreated Follicular Lymphoma</t>
+          <t>MO40597</t>
         </is>
       </c>
     </row>
@@ -1232,32 +832,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Hoffmann-La Roche</t>
+          <t>COVACTA</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>COVID</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>COVACTA</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Tocilizumab in Patients With Severe COVID-19 Pneumonia</t>
+          <t>WA42380</t>
         </is>
       </c>
     </row>
@@ -1272,29 +852,9 @@
           <t>Sanofi_NCT03637764_Oncology</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Sanofi</t>
-        </is>
-      </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Oncology</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Phase 1/Phase 2</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Terminated</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Isatuximab +/- Atezolizumab in Advanced Malignancies</t>
+          <t>ACT15377</t>
         </is>
       </c>
     </row>
@@ -1309,29 +869,9 @@
           <t>Tesaro_NCT01847274_Oncology</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Tesaro</t>
-        </is>
-      </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Oncology</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Niraparib vs Placebo Maintenance in Platinum Sensitive Ovarian Cancer</t>
+          <t>PR-30-5011-C</t>
         </is>
       </c>
     </row>
@@ -1346,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1357,15 +897,10 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>study_code</t>
+          <t>soa_pages</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
-        <is>
-          <t>soa_pages</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
         <is>
           <t>protocol_url</t>
         </is>
@@ -1379,15 +914,10 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>OPINION</t>
+          <t>40-44</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
-        <is>
-          <t>40-44</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/41/NCT03402841/Prot_002.pdf</t>
         </is>
@@ -1399,12 +929,12 @@
           <t>NCT04573309</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>14-17</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
-        <is>
-          <t>14-17</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/09/NCT04573309/Prot_000.pdf</t>
         </is>
@@ -1416,12 +946,12 @@
           <t>NCT03283098</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>32-36</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
-        <is>
-          <t>32-36</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/98/NCT03283098/Prot_001.pdf</t>
         </is>
@@ -1435,15 +965,10 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PIVOT IO 020</t>
+          <t>28-42</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
-        <is>
-          <t>28-42</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/49/NCT04730349/Prot_SAP_000.pdf</t>
         </is>
@@ -1457,15 +982,10 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MONARCH 2</t>
+          <t>73-78</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
-        <is>
-          <t>73-78</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/03/NCT02107703/Prot_000.pdf</t>
         </is>
@@ -1477,12 +997,12 @@
           <t>NCT03421379</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>11-18</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
-        <is>
-          <t>11-18</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/79/NCT03421379/Prot_000.pdf</t>
         </is>
@@ -1494,12 +1014,12 @@
           <t>NCT04004988</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10-11</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
-        <is>
-          <t>10-11</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/88/NCT04004988/Prot_000.pdf</t>
         </is>
@@ -1513,15 +1033,10 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SURMOUNT-1</t>
+          <t>18-24</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
-        <is>
-          <t>18-24</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/22/NCT04184622/Prot_000.pdf</t>
         </is>
@@ -1533,12 +1048,12 @@
           <t>NCT04557384</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>16-24</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
-        <is>
-          <t>16-24</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/84/NCT04557384/Prot_000.pdf</t>
         </is>
@@ -1552,15 +1067,10 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>INSTRUCT-UC</t>
+          <t>17-46</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
-        <is>
-          <t>17-46</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/79/NCT04677179/Prot_000.pdf</t>
         </is>
@@ -1572,12 +1082,12 @@
           <t>NCT05176314</t>
         </is>
       </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>10-11</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
-        <is>
-          <t>10-11</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/14/NCT05176314/Prot_000.pdf</t>
         </is>
@@ -1589,12 +1099,12 @@
           <t>NCT05324124</t>
         </is>
       </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
-        <is>
-          <t>9-12</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/24/NCT05324124/Prot_000.pdf</t>
         </is>
@@ -1606,7 +1116,7 @@
           <t>NCT03523273</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/73/NCT03523273/Prot_SAP_000.pdf</t>
         </is>
@@ -1618,12 +1128,12 @@
           <t>NCT05259917</t>
         </is>
       </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>17-18</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
-        <is>
-          <t>17-18</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/17/NCT05259917/Prot_000.pdf</t>
         </is>
@@ -1637,15 +1147,10 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>STEP 1</t>
+          <t>8-13</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
-        <is>
-          <t>8-13</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/35/NCT03548935/Prot_002.pdf</t>
         </is>
@@ -1659,15 +1164,10 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>STEP 4</t>
+          <t>8-11</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
-        <is>
-          <t>8-11</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/87/NCT03548987/Prot_000.pdf</t>
         </is>
@@ -1681,15 +1181,10 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>STEP 5</t>
+          <t>9-12</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
-        <is>
-          <t>9-12</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/30/NCT03693430/Prot_000.pdf</t>
         </is>
@@ -1703,15 +1198,10 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MODUL</t>
+          <t>169-193</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
-        <is>
-          <t>169-193</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/89/NCT02291289/Prot_000.pdf</t>
         </is>
@@ -1723,12 +1213,12 @@
           <t>NCT03817853</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>100-102</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
-        <is>
-          <t>100-102</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/53/NCT03817853/Prot_002.pdf</t>
         </is>
@@ -1742,15 +1232,10 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>COVACTA</t>
+          <t>77-85</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
-        <is>
-          <t>77-85</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/15/NCT04320615/Prot_000.pdf</t>
         </is>
@@ -1762,12 +1247,12 @@
           <t>NCT03637764</t>
         </is>
       </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>18-21</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
-        <is>
-          <t>18-21</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/64/NCT03637764/Prot_000.pdf</t>
         </is>
@@ -1779,12 +1264,12 @@
           <t>NCT01847274</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>63-78</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
-        <is>
-          <t>63-78</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
         <is>
           <t>https://ClinicalTrials.gov/ProvidedDocs/74/NCT01847274/Prot_000.pdf</t>
         </is>
@@ -1798,15 +1283,10 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>LZZT</t>
+          <t>53-54</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
-        <is>
-          <t>53-54</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/data4knowledge/usdm_data/main/source_data/protocols/CDISC_Pilot/CDISC_Pilot_Study.pdf</t>
         </is>

</xml_diff>

<commit_message>
Set therapeutic_area for the three blank-TA protocols; regenerate activity inventory
studies sheet gains a therapeutic_area column (overrides d4k_folder suffix,
code commit adc1695 in soa2usdm): NCT04677179 = Ulcerative Colitis (protocol
title page, J1P-MC-KFAH(b) INSTRUCT-UC); NCT05176314 and NCT05324124 =
ClinPharm (Phase 1 healthy-participant DDI / food-effect studies).

Inventory regenerated: 899 consolidated / 1206 source rows — the +18 source
rows are NCT04677179's Table 4 rework from earlier today flowing through
(consolidated count unchanged).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ngh7vdHGtu1NyYykSUYVx2
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -438,6 +438,11 @@
           <t>study_code</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>therapeutic_area</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -650,6 +655,11 @@
           <t>J1P-MC-KFAH</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Ulcerative Colitis</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -667,6 +677,11 @@
           <t>J2N-MC-JZNW</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ClinPharm</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -682,6 +697,11 @@
       <c r="D14" t="inlineStr">
         <is>
           <t>J2G-MC-JZPA</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ClinPharm</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Declare NCT03523273 not extractable; regenerate both indexes
NCT03523273 (Inv_NCT03523273_Weight) is row 23 of the studies sheet but its
posted protocol contains no SoA table, so it can never be extracted. It was
being reported as "1 pending" on the published index -- outstanding work
that will never be done.

studies_protocols.xlsx gains an excluded_reason column on the studies
sheet, set for this one study. All pre-existing rows and columns are
unchanged.

Both indexes regenerated against soa2usdm fb58085. The collection index
now reads 22 protocols | 22 processed | 0 pending | 1 excluded, with
NCT03523273 shown as "Not extractable -- posted protocol contains no SoA
table" rather than as a pending row. The root index card reads 22
protocols / 22 processed to match.

The corpus itself is unchanged; this is metadata and presentation only.
The re-extraction sweep scope is therefore 22 studies / 45 tables.
</commit_message>
<xml_diff>
--- a/collections/usdm_data/studies_protocols.xlsx
+++ b/collections/usdm_data/studies_protocols.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,6 +443,11 @@
           <t>therapeutic_area</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>excluded_reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -714,6 +719,11 @@
       <c r="B15" t="inlineStr">
         <is>
           <t>Inv_NCT03523273_Weight</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>posted protocol contains no SoA table</t>
         </is>
       </c>
     </row>

</xml_diff>